<commit_message>
Pre-submission revisions: manuscript, figures notebook, bibliography, data fixes
</commit_message>
<xml_diff>
--- a/data/misc./mixed_in_special_election_candidates.xlsx
+++ b/data/misc./mixed_in_special_election_candidates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdpruett/Desktop/CES Accuracy Analysis/data/misc./"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdpruett/Repos/CES Accuracy Analysis/data/misc./"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5B5C5B2-BBB5-234E-8EFE-4B8B125F67FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56572FEB-4122-6942-A300-A904918AC2DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2240" yWindow="660" windowWidth="23100" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40200" yWindow="140" windowWidth="23100" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1659" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1647" uniqueCount="453">
   <si>
     <t>state</t>
   </si>
@@ -1346,15 +1346,6 @@
   </si>
   <si>
     <t>Washington</t>
-  </si>
-  <si>
-    <t>Washington Secretary of State</t>
-  </si>
-  <si>
-    <t>Steve Hobbs</t>
-  </si>
-  <si>
-    <t>Julie Anderson</t>
   </si>
   <si>
     <t>Washington State Senate District 27</t>
@@ -1748,7 +1739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H277"/>
+  <dimension ref="A1:H275"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
@@ -1757,7 +1748,7 @@
     <col min="5" max="5" width="32.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -8712,10 +8703,10 @@
         <v>443</v>
       </c>
       <c r="E269" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F269">
-        <v>1468521</v>
+        <v>17074</v>
       </c>
       <c r="G269" t="s">
         <v>12</v>
@@ -8738,10 +8729,10 @@
         <v>444</v>
       </c>
       <c r="E270" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F270">
-        <v>1351926</v>
+        <v>41035</v>
       </c>
       <c r="G270" t="s">
         <v>12</v>
@@ -8755,7 +8746,7 @@
         <v>441</v>
       </c>
       <c r="B271">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C271" t="s">
         <v>445</v>
@@ -8767,7 +8758,7 @@
         <v>16</v>
       </c>
       <c r="F271">
-        <v>17074</v>
+        <v>27818</v>
       </c>
       <c r="G271" t="s">
         <v>12</v>
@@ -8781,7 +8772,7 @@
         <v>441</v>
       </c>
       <c r="B272">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="C272" t="s">
         <v>445</v>
@@ -8793,7 +8784,7 @@
         <v>11</v>
       </c>
       <c r="F272">
-        <v>41035</v>
+        <v>39799</v>
       </c>
       <c r="G272" t="s">
         <v>12</v>
@@ -8804,22 +8795,22 @@
     </row>
     <row r="273" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A273" s="2" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="B273">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="C273" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D273" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E273" t="s">
         <v>16</v>
       </c>
       <c r="F273">
-        <v>27818</v>
+        <v>9909</v>
       </c>
       <c r="G273" t="s">
         <v>12</v>
@@ -8830,22 +8821,22 @@
     </row>
     <row r="274" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A274" s="2" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="B274">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="C274" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D274" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E274" t="s">
         <v>11</v>
       </c>
       <c r="F274">
-        <v>39799</v>
+        <v>12249</v>
       </c>
       <c r="G274" t="s">
         <v>12</v>
@@ -8856,79 +8847,27 @@
     </row>
     <row r="275" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A275" s="2" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="B275">
         <v>2018</v>
       </c>
       <c r="C275" t="s">
+        <v>449</v>
+      </c>
+      <c r="D275" t="s">
         <v>452</v>
       </c>
-      <c r="D275" t="s">
-        <v>453</v>
-      </c>
       <c r="E275" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="F275">
-        <v>9909</v>
+        <v>273</v>
       </c>
       <c r="G275" t="s">
         <v>12</v>
       </c>
       <c r="H275" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="276" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A276" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="B276">
-        <v>2018</v>
-      </c>
-      <c r="C276" t="s">
-        <v>452</v>
-      </c>
-      <c r="D276" t="s">
-        <v>454</v>
-      </c>
-      <c r="E276" t="s">
-        <v>11</v>
-      </c>
-      <c r="F276">
-        <v>12249</v>
-      </c>
-      <c r="G276" t="s">
-        <v>12</v>
-      </c>
-      <c r="H276" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="277" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A277" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="B277">
-        <v>2018</v>
-      </c>
-      <c r="C277" t="s">
-        <v>452</v>
-      </c>
-      <c r="D277" t="s">
-        <v>455</v>
-      </c>
-      <c r="E277" t="s">
-        <v>80</v>
-      </c>
-      <c r="F277">
-        <v>273</v>
-      </c>
-      <c r="G277" t="s">
-        <v>12</v>
-      </c>
-      <c r="H277" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>